<commit_message>
feat(modelo): consolidacion directa con posiciones finitas (fase 7)
Co-Authored-By: Daniel mazzucco <mazzuccoda@gmail.com>
</commit_message>
<xml_diff>
--- a/datos/entrada_ejemplo.xlsx
+++ b/datos/entrada_ejemplo.xlsx
@@ -1873,7 +1873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1912,6 +1912,16 @@
           <t>capacidad_diaria_tn</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>posiciones_consolidacion</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>contenedores_por_posicion_dia</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1941,6 +1951,12 @@
       <c r="G2" t="n">
         <v>0</v>
       </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1965,11 +1981,17 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1994,11 +2016,17 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2023,11 +2051,17 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2052,11 +2086,17 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2081,11 +2121,17 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2115,6 +2161,12 @@
       <c r="G8" t="n">
         <v>500</v>
       </c>
+      <c r="H8" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2143,6 +2195,12 @@
       </c>
       <c r="G9" t="n">
         <v>600</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -3605,7 +3663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3628,7 +3686,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ZARATE</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3637,13 +3695,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ZARATE</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3652,13 +3710,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ZARATE</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3667,13 +3725,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3682,13 +3740,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3697,21 +3755,246 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>NORRY</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BOREAS</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BOREAS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BOREAS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RUTA9</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RUTA9</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RUTA9</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DODERO</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DODERO</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DODERO</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ZARATE</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ZARATE</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ZARATE</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>T4</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ACEITE</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(modelo): cross docking con cupo diario por sitio y sin almacenaje (fase 8)
Co-Authored-By: Daniel mazzucco <mazzuccoda@gmail.com>
</commit_message>
<xml_diff>
--- a/datos/entrada_ejemplo.xlsx
+++ b/datos/entrada_ejemplo.xlsx
@@ -1873,7 +1873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1922,6 +1922,11 @@
           <t>contenedores_por_posicion_dia</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>posiciones_cross_dock</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1957,6 +1962,9 @@
       <c r="I2" t="n">
         <v>0</v>
       </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1992,6 +2000,9 @@
       <c r="I3" t="n">
         <v>4</v>
       </c>
+      <c r="J3" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2027,6 +2038,9 @@
       <c r="I4" t="n">
         <v>4</v>
       </c>
+      <c r="J4" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2062,6 +2076,9 @@
       <c r="I5" t="n">
         <v>3</v>
       </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2097,6 +2114,9 @@
       <c r="I6" t="n">
         <v>3</v>
       </c>
+      <c r="J6" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2132,6 +2152,9 @@
       <c r="I7" t="n">
         <v>3</v>
       </c>
+      <c r="J7" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2167,6 +2190,9 @@
       <c r="I8" t="n">
         <v>8</v>
       </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2201,6 +2227,9 @@
       </c>
       <c r="I9" t="n">
         <v>8</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3663,7 +3692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3679,6 +3708,11 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>tipo_servicio</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>tarifa_usd_tn</t>
         </is>
       </c>
@@ -3694,7 +3728,12 @@
           <t>JUGO</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3706,10 +3745,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CASCARA</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -3721,47 +3765,62 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ACEITE</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>14</v>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>JUGO</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>10</v>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CASCARA</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>8</v>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3769,14 +3828,19 @@
           <t>ACEITE</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>13</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3784,74 +3848,99 @@
           <t>JUGO</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>8</v>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CASCARA</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>7</v>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ACEITE</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>15</v>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JUGO</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>11</v>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CASCARA</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>9</v>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3859,14 +3948,19 @@
           <t>ACEITE</t>
         </is>
       </c>
-      <c r="C13" t="n">
-        <v>12</v>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DODERO</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3874,74 +3968,99 @@
           <t>JUGO</t>
         </is>
       </c>
-      <c r="C14" t="n">
-        <v>9</v>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DODERO</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CASCARA</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>8</v>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DODERO</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ACEITE</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>14</v>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ZARATE</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>JUGO</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>12</v>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ZARATE</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CASCARA</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>10</v>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ZARATE</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3949,14 +4068,19 @@
           <t>ACEITE</t>
         </is>
       </c>
-      <c r="C19" t="n">
-        <v>18</v>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>RUTA9</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3964,37 +4088,352 @@
           <t>JUGO</t>
         </is>
       </c>
-      <c r="C20" t="n">
-        <v>15</v>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>RUTA9</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CASCARA</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>11</v>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>RUTA9</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>RUTA9</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>RUTA9</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>RUTA9</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DODERO</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DODERO</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DODERO</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DODERO</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DODERO</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>DODERO</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CROSS_DOCK</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ZARATE</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ZARATE</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ZARATE</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>T4</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>ACEITE</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(modelo): la flota de producto se consume como capacidad diaria (ADR-044)
Los viajes planta-deposito y los de cross dock toman camion-dia, el pool del
flujo pasa a ser la flota de portacontenedores y el flete se cobra por viaje.
Con esto E-01 y E-02 dejan de ser identicos a E-00: el barrido responde
cuantos camiones hacen falta.

Co-Authored-By: Daniel mazzucco <mazzuccoda@gmail.com>
</commit_message>
<xml_diff>
--- a/datos/entrada_ejemplo.xlsx
+++ b/datos/entrada_ejemplo.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,40 +473,60 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>camiones_portacontenedor</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>capacidad_camion_tn</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>velocidad_camion_kmh</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>horas_operativas_dia</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>factor_produccion</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>factor_capacidad_planta</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>factor_capacidad_deposito</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>factor_storage</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>ventana_demanda</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>habilita_cross_dock</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>deterministico</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>estrategia_consolidacion</t>
         </is>
@@ -540,34 +560,46 @@
         <v>15</v>
       </c>
       <c r="I2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="L2" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N2" t="n">
         <v>1</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S2" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
@@ -601,34 +633,46 @@
         <v>15</v>
       </c>
       <c r="I3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
@@ -662,34 +706,46 @@
         <v>15</v>
       </c>
       <c r="I4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="M4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
@@ -723,34 +779,46 @@
         <v>15</v>
       </c>
       <c r="I5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="L5" t="n">
-        <v>0.5</v>
+        <v>70</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N5" t="n">
         <v>1</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>1</v>
+      </c>
+      <c r="R5" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
@@ -784,34 +852,46 @@
         <v>15</v>
       </c>
       <c r="I6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="L6" t="n">
-        <v>2</v>
+        <v>70</v>
       </c>
       <c r="M6" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N6" t="n">
         <v>1</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S6" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
@@ -845,34 +925,46 @@
         <v>15</v>
       </c>
       <c r="I7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="L7" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="M7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N7" t="n">
         <v>1</v>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
@@ -906,34 +998,46 @@
         <v>15</v>
       </c>
       <c r="I8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J8" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" t="n">
+        <v>25</v>
+      </c>
+      <c r="L8" t="n">
+        <v>70</v>
+      </c>
+      <c r="M8" t="n">
+        <v>10</v>
+      </c>
+      <c r="N8" t="n">
         <v>1.3</v>
       </c>
-      <c r="K8" t="n">
+      <c r="O8" t="n">
         <v>1</v>
       </c>
-      <c r="L8" t="n">
+      <c r="P8" t="n">
         <v>1</v>
       </c>
-      <c r="M8" t="n">
+      <c r="Q8" t="n">
         <v>1</v>
       </c>
-      <c r="N8" t="n">
+      <c r="R8" t="n">
         <v>1</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
@@ -967,34 +1071,46 @@
         <v>15</v>
       </c>
       <c r="I9" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" t="n">
+        <v>25</v>
+      </c>
+      <c r="L9" t="n">
+        <v>70</v>
+      </c>
+      <c r="M9" t="n">
+        <v>10</v>
+      </c>
+      <c r="N9" t="n">
         <v>0.7</v>
       </c>
-      <c r="K9" t="n">
+      <c r="O9" t="n">
         <v>1</v>
       </c>
-      <c r="L9" t="n">
+      <c r="P9" t="n">
         <v>1</v>
       </c>
-      <c r="M9" t="n">
+      <c r="Q9" t="n">
         <v>1</v>
       </c>
-      <c r="N9" t="n">
+      <c r="R9" t="n">
         <v>1</v>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
@@ -1028,34 +1144,46 @@
         <v>15</v>
       </c>
       <c r="I10" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J10" t="n">
+        <v>4</v>
+      </c>
+      <c r="K10" t="n">
+        <v>25</v>
+      </c>
+      <c r="L10" t="n">
+        <v>70</v>
+      </c>
+      <c r="M10" t="n">
+        <v>10</v>
+      </c>
+      <c r="N10" t="n">
         <v>1</v>
       </c>
-      <c r="K10" t="n">
+      <c r="O10" t="n">
         <v>1</v>
       </c>
-      <c r="L10" t="n">
+      <c r="P10" t="n">
         <v>1</v>
       </c>
-      <c r="M10" t="n">
+      <c r="Q10" t="n">
         <v>1</v>
       </c>
-      <c r="N10" t="n">
+      <c r="R10" t="n">
         <v>0.5</v>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
@@ -1089,34 +1217,46 @@
         <v>15</v>
       </c>
       <c r="I11" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K11" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="M11" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N11" t="n">
         <v>1</v>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
@@ -1150,34 +1290,46 @@
         <v>15</v>
       </c>
       <c r="I12" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K12" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="L12" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="M12" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="N12" t="n">
         <v>1</v>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O12" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>2</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
@@ -1211,34 +1363,46 @@
         <v>15</v>
       </c>
       <c r="I13" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K13" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="L13" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="M13" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N13" t="n">
         <v>1</v>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="O13" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>1</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>CONSOLIDACION_TERMINAL</t>
         </is>

</xml_diff>

<commit_message>
feat(modelo): lote comercial acumulativo (fase 2, ADR-047)
La produccion diaria entra como una capa nueva del mismo lote abierto en
lugar de crear una identidad comercial por dia. LoteProducto suma cliente,
calidad, toneladasObjetivo y estadoComercial; el lote se cierra cuando la
produccion acumulada alcanza el objetivo y el despacho parcial no lo cierra.

Los datos comerciales vienen del contrato, no del codigo: columna nueva
toneladas_objetivo_lote_tn en Producto, y cliente_default y calidad_default
en Escenario.

Verificado en PLE: build limpio, campania completa sin excepciones, 360
corridas Finished, misma corrida desde Excel y sintetico.

Co-Authored-By: Daniel mazzucco <mazzuccoda@gmail.com>
</commit_message>
<xml_diff>
--- a/datos/entrada_ejemplo.xlsx
+++ b/datos/entrada_ejemplo.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,6 +531,16 @@
           <t>estrategia_consolidacion</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>cliente_default</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>calidad_default</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -604,6 +614,16 @@
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -677,6 +697,16 @@
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
       </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -750,6 +780,16 @@
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
       </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -823,6 +863,16 @@
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
       </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -896,6 +946,16 @@
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
       </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -969,6 +1029,16 @@
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
       </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1042,6 +1112,16 @@
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
       </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1115,6 +1195,16 @@
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
       </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1188,6 +1278,16 @@
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
       </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1261,6 +1361,16 @@
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
       </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1334,6 +1444,16 @@
           <t>CONSOLIDACION_DEPOSITO</t>
         </is>
       </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1405,6 +1525,16 @@
       <c r="U13" t="inlineStr">
         <is>
           <t>CONSOLIDACION_TERMINAL</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
         </is>
       </c>
     </row>
@@ -2710,7 +2840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2729,6 +2859,11 @@
           <t>capacidad_contenedor_tn</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>toneladas_objetivo_lote_tn</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2744,6 +2879,9 @@
       <c r="C2" t="n">
         <v>25</v>
       </c>
+      <c r="D2" t="n">
+        <v>2000</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2759,6 +2897,9 @@
       <c r="C3" t="n">
         <v>25</v>
       </c>
+      <c r="D3" t="n">
+        <v>1200</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2773,6 +2914,9 @@
       </c>
       <c r="C4" t="n">
         <v>20</v>
+      </c>
+      <c r="D4" t="n">
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(modelo): flujo fisico con los cuatro circuitos (fase 21, ADR-050)
Co-Authored-By: Daniel mazzucco <mazzuccoda@gmail.com>
</commit_message>
<xml_diff>
--- a/datos/entrada_ejemplo.xlsx
+++ b/datos/entrada_ejemplo.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB14"/>
+  <dimension ref="A1:AB15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1864,6 +1864,106 @@
       <c r="AB14" t="inlineStr">
         <is>
           <t>REACTIVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>E-13</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>183</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F15" t="n">
+        <v>40</v>
+      </c>
+      <c r="G15" t="n">
+        <v>400</v>
+      </c>
+      <c r="H15" t="n">
+        <v>15</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K15" t="n">
+        <v>25</v>
+      </c>
+      <c r="L15" t="n">
+        <v>70</v>
+      </c>
+      <c r="M15" t="n">
+        <v>10</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_PLANTA</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X15" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
         </is>
       </c>
     </row>
@@ -3326,19 +3426,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -3901,7 +4001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3999,7 +4099,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FRINOA</t>
+          <t>PLANTA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4008,13 +4108,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4023,13 +4123,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4038,13 +4138,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4053,13 +4153,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>80</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DODERO</t>
+          <t>RUTA9</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4068,28 +4168,28 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>130</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FRINOA</t>
+          <t>DODERO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>ZARATE</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>PLANTA</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4098,13 +4198,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>110</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4113,13 +4213,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>90</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4128,21 +4228,51 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>160</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>BOREAS</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>RUTA9</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>DODERO</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>T4</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C18" t="n">
         <v>70</v>
       </c>
     </row>
@@ -4576,7 +4706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4604,7 +4734,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FRINOA</t>
+          <t>PLANTA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4618,13 +4748,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FRINOA</t>
+          <t>PLANTA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4638,13 +4768,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FRINOA</t>
+          <t>PLANTA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4658,13 +4788,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4678,13 +4808,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4698,13 +4828,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4718,13 +4848,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4738,13 +4868,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4758,13 +4888,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4778,13 +4908,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4798,13 +4928,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4818,13 +4948,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4838,13 +4968,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DODERO</t>
+          <t>RUTA9</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4858,13 +4988,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DODERO</t>
+          <t>RUTA9</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4878,13 +5008,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DODERO</t>
+          <t>RUTA9</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -4898,18 +5028,18 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FRINOA</t>
+          <t>DODERO</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>ZARATE</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -4918,18 +5048,18 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FRINOA</t>
+          <t>DODERO</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>ZARATE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -4938,18 +5068,18 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FRINOA</t>
+          <t>DODERO</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>ZARATE</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -4958,13 +5088,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>PLANTA</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4978,13 +5108,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>PLANTA</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4998,13 +5128,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>PLANTA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5018,13 +5148,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5038,13 +5168,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5058,13 +5188,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5078,13 +5208,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5098,13 +5228,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5118,13 +5248,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5138,13 +5268,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DODERO</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5158,13 +5288,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DODERO</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5178,26 +5308,146 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>BOREAS</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>RUTA9</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>RUTA9</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>RUTA9</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>DODERO</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>T4</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>ACEITE</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DODERO</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>DODERO</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
         <v>7</v>
       </c>
     </row>
@@ -5212,7 +5462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5240,7 +5490,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FRINOA</t>
+          <t>PLANTA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5260,17 +5510,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FRINOA</t>
+          <t>PLANTA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>JUGO</t>
+          <t>CASCARA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -5280,12 +5530,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FRINOA</t>
+          <t>PLANTA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CASCARA</t>
+          <t>ACEITE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -5294,7 +5544,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -5305,16 +5555,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CASCARA</t>
+          <t>JUGO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -5325,16 +5575,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ACEITE</t>
+          <t>JUGO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -5345,76 +5595,76 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ACEITE</t>
+          <t>CASCARA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>JUGO</t>
+          <t>CASCARA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>JUGO</t>
+          <t>ACEITE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NORRY</t>
+          <t>FRINOA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CASCARA</t>
+          <t>ACEITE</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11">
@@ -5425,16 +5675,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CASCARA</t>
+          <t>JUGO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -5445,16 +5695,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ACEITE</t>
+          <t>JUGO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -5465,76 +5715,76 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ACEITE</t>
+          <t>CASCARA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JUGO</t>
+          <t>CASCARA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>JUGO</t>
+          <t>ACEITE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BOREAS</t>
+          <t>NORRY</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CASCARA</t>
+          <t>ACEITE</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
@@ -5545,16 +5795,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CASCARA</t>
+          <t>JUGO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18">
@@ -5565,16 +5815,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ACEITE</t>
+          <t>JUGO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
@@ -5585,76 +5835,76 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ACEITE</t>
+          <t>CASCARA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>JUGO</t>
+          <t>CASCARA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>JUGO</t>
+          <t>ACEITE</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RUTA9</t>
+          <t>BOREAS</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CASCARA</t>
+          <t>ACEITE</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23">
@@ -5665,16 +5915,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CASCARA</t>
+          <t>JUGO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24">
@@ -5685,16 +5935,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ACEITE</t>
+          <t>JUGO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
@@ -5705,76 +5955,76 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ACEITE</t>
+          <t>CASCARA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DODERO</t>
+          <t>RUTA9</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>JUGO</t>
+          <t>CASCARA</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>DODERO</t>
+          <t>RUTA9</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>JUGO</t>
+          <t>ACEITE</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DODERO</t>
+          <t>RUTA9</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CASCARA</t>
+          <t>ACEITE</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29">
@@ -5785,16 +6035,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CASCARA</t>
+          <t>JUGO</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30">
@@ -5805,16 +6055,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ACEITE</t>
+          <t>JUGO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31">
@@ -5825,47 +6075,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ACEITE</t>
+          <t>CASCARA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CROSS_DOCK</t>
+          <t>CONSOLIDACION</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ZARATE</t>
+          <t>DODERO</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>JUGO</t>
+          <t>CASCARA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ZARATE</t>
+          <t>DODERO</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CASCARA</t>
+          <t>ACEITE</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5874,13 +6124,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ZARATE</t>
+          <t>DODERO</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5890,17 +6140,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CONSOLIDACION</t>
+          <t>CROSS_DOCK</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>ZARATE</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5914,13 +6164,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>ZARATE</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5934,26 +6184,86 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>ZARATE</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>T4</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>ACEITE</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>JUGO</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
         <is>
           <t>CONSOLIDACION</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D38" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>CASCARA</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(modelo): evaluador de circuitos por pedido y escenarios economicos (C5+C6, ADR-054)
Co-Authored-By: Daniel mazzucco <mazzuccoda@gmail.com>
</commit_message>
<xml_diff>
--- a/datos/entrada_ejemplo.xlsx
+++ b/datos/entrada_ejemplo.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB15"/>
+  <dimension ref="A1:AK37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -567,6 +567,51 @@
           <t>politica_frio_propio</t>
         </is>
       </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>politica_seleccion</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>servicio_minimo_proyectado</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>factor_tarifa_flete</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>factor_tarifa_round_trip</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>factor_tarifa_cross_dock</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>factor_tarifa_terminal</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>factor_consolidacion_planta</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>factor_cupo_cross_dock</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>factor_capacidad_terminal</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -667,6 +712,35 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -767,6 +841,35 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -867,6 +970,35 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD4" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -967,6 +1099,35 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1067,6 +1228,35 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1167,6 +1357,35 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>FIJA_CROSS_DOCK_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD7" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1267,6 +1486,35 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1367,6 +1615,35 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD9" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1467,6 +1744,35 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD10" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1567,6 +1873,35 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD11" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1667,6 +2002,35 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD12" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1767,6 +2131,35 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>FIJA_CROSS_DOCK_TERMINAL</t>
+        </is>
+      </c>
+      <c r="AD13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1867,6 +2260,35 @@
           <t>REACTIVA</t>
         </is>
       </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD14" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1966,6 +2388,2873 @@
         <is>
           <t>FLEXIBLE</t>
         </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>FIJA_PLANTA</t>
+        </is>
+      </c>
+      <c r="AD15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>E-14</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>183</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>40</v>
+      </c>
+      <c r="G16" t="n">
+        <v>400</v>
+      </c>
+      <c r="H16" t="n">
+        <v>15</v>
+      </c>
+      <c r="I16" t="n">
+        <v>3</v>
+      </c>
+      <c r="J16" t="n">
+        <v>4</v>
+      </c>
+      <c r="K16" t="n">
+        <v>25</v>
+      </c>
+      <c r="L16" t="n">
+        <v>70</v>
+      </c>
+      <c r="M16" t="n">
+        <v>10</v>
+      </c>
+      <c r="N16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" t="n">
+        <v>1</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
+      <c r="R16" t="n">
+        <v>1</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X16" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>MENOR_COSTO_INCREMENTAL_FACTIBLE</t>
+        </is>
+      </c>
+      <c r="AD16" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>E-15</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>183</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>40</v>
+      </c>
+      <c r="G17" t="n">
+        <v>400</v>
+      </c>
+      <c r="H17" t="n">
+        <v>15</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3</v>
+      </c>
+      <c r="J17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" t="n">
+        <v>25</v>
+      </c>
+      <c r="L17" t="n">
+        <v>70</v>
+      </c>
+      <c r="M17" t="n">
+        <v>10</v>
+      </c>
+      <c r="N17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>1</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X17" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>MENOR_COSTO_END_TO_END_FACTIBLE</t>
+        </is>
+      </c>
+      <c r="AD17" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>E-16</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>183</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F18" t="n">
+        <v>40</v>
+      </c>
+      <c r="G18" t="n">
+        <v>400</v>
+      </c>
+      <c r="H18" t="n">
+        <v>15</v>
+      </c>
+      <c r="I18" t="n">
+        <v>3</v>
+      </c>
+      <c r="J18" t="n">
+        <v>4</v>
+      </c>
+      <c r="K18" t="n">
+        <v>25</v>
+      </c>
+      <c r="L18" t="n">
+        <v>70</v>
+      </c>
+      <c r="M18" t="n">
+        <v>10</v>
+      </c>
+      <c r="N18" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>1</v>
+      </c>
+      <c r="R18" t="n">
+        <v>1</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X18" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>PRIORIDAD_FRIO_PROPIO</t>
+        </is>
+      </c>
+      <c r="AD18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>E-17</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>183</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F19" t="n">
+        <v>40</v>
+      </c>
+      <c r="G19" t="n">
+        <v>400</v>
+      </c>
+      <c r="H19" t="n">
+        <v>15</v>
+      </c>
+      <c r="I19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J19" t="n">
+        <v>4</v>
+      </c>
+      <c r="K19" t="n">
+        <v>25</v>
+      </c>
+      <c r="L19" t="n">
+        <v>70</v>
+      </c>
+      <c r="M19" t="n">
+        <v>10</v>
+      </c>
+      <c r="N19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X19" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>MENOR_COSTO_INCREMENTAL_FACTIBLE</t>
+        </is>
+      </c>
+      <c r="AD19" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>E-18</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>183</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F20" t="n">
+        <v>40</v>
+      </c>
+      <c r="G20" t="n">
+        <v>400</v>
+      </c>
+      <c r="H20" t="n">
+        <v>15</v>
+      </c>
+      <c r="I20" t="n">
+        <v>3</v>
+      </c>
+      <c r="J20" t="n">
+        <v>4</v>
+      </c>
+      <c r="K20" t="n">
+        <v>25</v>
+      </c>
+      <c r="L20" t="n">
+        <v>70</v>
+      </c>
+      <c r="M20" t="n">
+        <v>10</v>
+      </c>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
+      <c r="O20" t="n">
+        <v>1</v>
+      </c>
+      <c r="P20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>1</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X20" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD20" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>E-19</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>183</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F21" t="n">
+        <v>40</v>
+      </c>
+      <c r="G21" t="n">
+        <v>400</v>
+      </c>
+      <c r="H21" t="n">
+        <v>15</v>
+      </c>
+      <c r="I21" t="n">
+        <v>3</v>
+      </c>
+      <c r="J21" t="n">
+        <v>4</v>
+      </c>
+      <c r="K21" t="n">
+        <v>25</v>
+      </c>
+      <c r="L21" t="n">
+        <v>70</v>
+      </c>
+      <c r="M21" t="n">
+        <v>10</v>
+      </c>
+      <c r="N21" t="n">
+        <v>1</v>
+      </c>
+      <c r="O21" t="n">
+        <v>1</v>
+      </c>
+      <c r="P21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>1</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X21" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD21" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>E-20</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>183</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>40</v>
+      </c>
+      <c r="G22" t="n">
+        <v>400</v>
+      </c>
+      <c r="H22" t="n">
+        <v>15</v>
+      </c>
+      <c r="I22" t="n">
+        <v>3</v>
+      </c>
+      <c r="J22" t="n">
+        <v>4</v>
+      </c>
+      <c r="K22" t="n">
+        <v>25</v>
+      </c>
+      <c r="L22" t="n">
+        <v>70</v>
+      </c>
+      <c r="M22" t="n">
+        <v>10</v>
+      </c>
+      <c r="N22" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>1</v>
+      </c>
+      <c r="P22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>1</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X22" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD22" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>E-21</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>183</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>40</v>
+      </c>
+      <c r="G23" t="n">
+        <v>400</v>
+      </c>
+      <c r="H23" t="n">
+        <v>15</v>
+      </c>
+      <c r="I23" t="n">
+        <v>3</v>
+      </c>
+      <c r="J23" t="n">
+        <v>4</v>
+      </c>
+      <c r="K23" t="n">
+        <v>25</v>
+      </c>
+      <c r="L23" t="n">
+        <v>70</v>
+      </c>
+      <c r="M23" t="n">
+        <v>10</v>
+      </c>
+      <c r="N23" t="n">
+        <v>1</v>
+      </c>
+      <c r="O23" t="n">
+        <v>1</v>
+      </c>
+      <c r="P23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>1</v>
+      </c>
+      <c r="R23" t="n">
+        <v>1</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X23" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD23" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>E-22</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>183</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F24" t="n">
+        <v>40</v>
+      </c>
+      <c r="G24" t="n">
+        <v>400</v>
+      </c>
+      <c r="H24" t="n">
+        <v>15</v>
+      </c>
+      <c r="I24" t="n">
+        <v>3</v>
+      </c>
+      <c r="J24" t="n">
+        <v>4</v>
+      </c>
+      <c r="K24" t="n">
+        <v>25</v>
+      </c>
+      <c r="L24" t="n">
+        <v>70</v>
+      </c>
+      <c r="M24" t="n">
+        <v>10</v>
+      </c>
+      <c r="N24" t="n">
+        <v>1</v>
+      </c>
+      <c r="O24" t="n">
+        <v>1</v>
+      </c>
+      <c r="P24" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>1</v>
+      </c>
+      <c r="R24" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X24" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>FIJA_CROSS_DOCK_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD24" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>E-23</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>183</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F25" t="n">
+        <v>40</v>
+      </c>
+      <c r="G25" t="n">
+        <v>400</v>
+      </c>
+      <c r="H25" t="n">
+        <v>15</v>
+      </c>
+      <c r="I25" t="n">
+        <v>3</v>
+      </c>
+      <c r="J25" t="n">
+        <v>4</v>
+      </c>
+      <c r="K25" t="n">
+        <v>25</v>
+      </c>
+      <c r="L25" t="n">
+        <v>70</v>
+      </c>
+      <c r="M25" t="n">
+        <v>10</v>
+      </c>
+      <c r="N25" t="n">
+        <v>1</v>
+      </c>
+      <c r="O25" t="n">
+        <v>1</v>
+      </c>
+      <c r="P25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>1</v>
+      </c>
+      <c r="R25" t="n">
+        <v>1</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X25" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>FIJA_CROSS_DOCK_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD25" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>E-24</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>183</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F26" t="n">
+        <v>40</v>
+      </c>
+      <c r="G26" t="n">
+        <v>400</v>
+      </c>
+      <c r="H26" t="n">
+        <v>15</v>
+      </c>
+      <c r="I26" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" t="n">
+        <v>4</v>
+      </c>
+      <c r="K26" t="n">
+        <v>25</v>
+      </c>
+      <c r="L26" t="n">
+        <v>70</v>
+      </c>
+      <c r="M26" t="n">
+        <v>10</v>
+      </c>
+      <c r="N26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O26" t="n">
+        <v>1</v>
+      </c>
+      <c r="P26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>1</v>
+      </c>
+      <c r="R26" t="n">
+        <v>1</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X26" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD26" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>E-25</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>183</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>40</v>
+      </c>
+      <c r="G27" t="n">
+        <v>400</v>
+      </c>
+      <c r="H27" t="n">
+        <v>15</v>
+      </c>
+      <c r="I27" t="n">
+        <v>3</v>
+      </c>
+      <c r="J27" t="n">
+        <v>4</v>
+      </c>
+      <c r="K27" t="n">
+        <v>25</v>
+      </c>
+      <c r="L27" t="n">
+        <v>70</v>
+      </c>
+      <c r="M27" t="n">
+        <v>10</v>
+      </c>
+      <c r="N27" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" t="n">
+        <v>1</v>
+      </c>
+      <c r="P27" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>1</v>
+      </c>
+      <c r="R27" t="n">
+        <v>1</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X27" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD27" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>E-26</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>183</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>40</v>
+      </c>
+      <c r="G28" t="n">
+        <v>400</v>
+      </c>
+      <c r="H28" t="n">
+        <v>7</v>
+      </c>
+      <c r="I28" t="n">
+        <v>3</v>
+      </c>
+      <c r="J28" t="n">
+        <v>4</v>
+      </c>
+      <c r="K28" t="n">
+        <v>25</v>
+      </c>
+      <c r="L28" t="n">
+        <v>70</v>
+      </c>
+      <c r="M28" t="n">
+        <v>10</v>
+      </c>
+      <c r="N28" t="n">
+        <v>1</v>
+      </c>
+      <c r="O28" t="n">
+        <v>1</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>1</v>
+      </c>
+      <c r="R28" t="n">
+        <v>1</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X28" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD28" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>E-27</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>183</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>40</v>
+      </c>
+      <c r="G29" t="n">
+        <v>400</v>
+      </c>
+      <c r="H29" t="n">
+        <v>30</v>
+      </c>
+      <c r="I29" t="n">
+        <v>3</v>
+      </c>
+      <c r="J29" t="n">
+        <v>4</v>
+      </c>
+      <c r="K29" t="n">
+        <v>25</v>
+      </c>
+      <c r="L29" t="n">
+        <v>70</v>
+      </c>
+      <c r="M29" t="n">
+        <v>10</v>
+      </c>
+      <c r="N29" t="n">
+        <v>1</v>
+      </c>
+      <c r="O29" t="n">
+        <v>1</v>
+      </c>
+      <c r="P29" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>1</v>
+      </c>
+      <c r="R29" t="n">
+        <v>1</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X29" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD29" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>E-28</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>183</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>40</v>
+      </c>
+      <c r="G30" t="n">
+        <v>400</v>
+      </c>
+      <c r="H30" t="n">
+        <v>60</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3</v>
+      </c>
+      <c r="J30" t="n">
+        <v>4</v>
+      </c>
+      <c r="K30" t="n">
+        <v>25</v>
+      </c>
+      <c r="L30" t="n">
+        <v>70</v>
+      </c>
+      <c r="M30" t="n">
+        <v>10</v>
+      </c>
+      <c r="N30" t="n">
+        <v>1</v>
+      </c>
+      <c r="O30" t="n">
+        <v>1</v>
+      </c>
+      <c r="P30" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>1</v>
+      </c>
+      <c r="R30" t="n">
+        <v>1</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X30" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD30" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>E-32</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>183</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F31" t="n">
+        <v>40</v>
+      </c>
+      <c r="G31" t="n">
+        <v>400</v>
+      </c>
+      <c r="H31" t="n">
+        <v>15</v>
+      </c>
+      <c r="I31" t="n">
+        <v>3</v>
+      </c>
+      <c r="J31" t="n">
+        <v>4</v>
+      </c>
+      <c r="K31" t="n">
+        <v>25</v>
+      </c>
+      <c r="L31" t="n">
+        <v>70</v>
+      </c>
+      <c r="M31" t="n">
+        <v>10</v>
+      </c>
+      <c r="N31" t="n">
+        <v>1</v>
+      </c>
+      <c r="O31" t="n">
+        <v>1</v>
+      </c>
+      <c r="P31" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>1</v>
+      </c>
+      <c r="R31" t="n">
+        <v>1</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X31" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD31" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>E-33</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>183</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>40</v>
+      </c>
+      <c r="G32" t="n">
+        <v>400</v>
+      </c>
+      <c r="H32" t="n">
+        <v>45</v>
+      </c>
+      <c r="I32" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" t="n">
+        <v>4</v>
+      </c>
+      <c r="K32" t="n">
+        <v>25</v>
+      </c>
+      <c r="L32" t="n">
+        <v>70</v>
+      </c>
+      <c r="M32" t="n">
+        <v>10</v>
+      </c>
+      <c r="N32" t="n">
+        <v>1</v>
+      </c>
+      <c r="O32" t="n">
+        <v>1</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>1</v>
+      </c>
+      <c r="R32" t="n">
+        <v>1</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X32" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD32" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>E-29</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>183</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>40</v>
+      </c>
+      <c r="G33" t="n">
+        <v>400</v>
+      </c>
+      <c r="H33" t="n">
+        <v>15</v>
+      </c>
+      <c r="I33" t="n">
+        <v>3</v>
+      </c>
+      <c r="J33" t="n">
+        <v>4</v>
+      </c>
+      <c r="K33" t="n">
+        <v>25</v>
+      </c>
+      <c r="L33" t="n">
+        <v>70</v>
+      </c>
+      <c r="M33" t="n">
+        <v>10</v>
+      </c>
+      <c r="N33" t="n">
+        <v>1</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="P33" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>1</v>
+      </c>
+      <c r="R33" t="n">
+        <v>1</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X33" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD33" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>E-30</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>183</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F34" t="n">
+        <v>40</v>
+      </c>
+      <c r="G34" t="n">
+        <v>400</v>
+      </c>
+      <c r="H34" t="n">
+        <v>15</v>
+      </c>
+      <c r="I34" t="n">
+        <v>3</v>
+      </c>
+      <c r="J34" t="n">
+        <v>4</v>
+      </c>
+      <c r="K34" t="n">
+        <v>25</v>
+      </c>
+      <c r="L34" t="n">
+        <v>70</v>
+      </c>
+      <c r="M34" t="n">
+        <v>10</v>
+      </c>
+      <c r="N34" t="n">
+        <v>1</v>
+      </c>
+      <c r="O34" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P34" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>1</v>
+      </c>
+      <c r="R34" t="n">
+        <v>1</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X34" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA34" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>FIJA_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD34" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>E-31</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>183</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F35" t="n">
+        <v>40</v>
+      </c>
+      <c r="G35" t="n">
+        <v>400</v>
+      </c>
+      <c r="H35" t="n">
+        <v>15</v>
+      </c>
+      <c r="I35" t="n">
+        <v>3</v>
+      </c>
+      <c r="J35" t="n">
+        <v>4</v>
+      </c>
+      <c r="K35" t="n">
+        <v>25</v>
+      </c>
+      <c r="L35" t="n">
+        <v>70</v>
+      </c>
+      <c r="M35" t="n">
+        <v>10</v>
+      </c>
+      <c r="N35" t="n">
+        <v>1</v>
+      </c>
+      <c r="O35" t="n">
+        <v>1</v>
+      </c>
+      <c r="P35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>1</v>
+      </c>
+      <c r="R35" t="n">
+        <v>1</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_PLANTA</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X35" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>FIJA_PLANTA</t>
+        </is>
+      </c>
+      <c r="AD35" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>E-34</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>183</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F36" t="n">
+        <v>40</v>
+      </c>
+      <c r="G36" t="n">
+        <v>400</v>
+      </c>
+      <c r="H36" t="n">
+        <v>15</v>
+      </c>
+      <c r="I36" t="n">
+        <v>3</v>
+      </c>
+      <c r="J36" t="n">
+        <v>4</v>
+      </c>
+      <c r="K36" t="n">
+        <v>25</v>
+      </c>
+      <c r="L36" t="n">
+        <v>70</v>
+      </c>
+      <c r="M36" t="n">
+        <v>10</v>
+      </c>
+      <c r="N36" t="n">
+        <v>1</v>
+      </c>
+      <c r="O36" t="n">
+        <v>1</v>
+      </c>
+      <c r="P36" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>1</v>
+      </c>
+      <c r="R36" t="n">
+        <v>1</v>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X36" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>FIJA_CROSS_DOCK_DEPOSITO</t>
+        </is>
+      </c>
+      <c r="AD36" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AK36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>E-35</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>183</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F37" t="n">
+        <v>40</v>
+      </c>
+      <c r="G37" t="n">
+        <v>400</v>
+      </c>
+      <c r="H37" t="n">
+        <v>15</v>
+      </c>
+      <c r="I37" t="n">
+        <v>3</v>
+      </c>
+      <c r="J37" t="n">
+        <v>4</v>
+      </c>
+      <c r="K37" t="n">
+        <v>25</v>
+      </c>
+      <c r="L37" t="n">
+        <v>70</v>
+      </c>
+      <c r="M37" t="n">
+        <v>10</v>
+      </c>
+      <c r="N37" t="n">
+        <v>1</v>
+      </c>
+      <c r="O37" t="n">
+        <v>1</v>
+      </c>
+      <c r="P37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>1</v>
+      </c>
+      <c r="R37" t="n">
+        <v>1</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>CONSOLIDACION_TERMINAL</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>GENERICO</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>ESTANDAR</t>
+        </is>
+      </c>
+      <c r="X37" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>FLEXIBLE</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>FIJA_CROSS_DOCK_TERMINAL</t>
+        </is>
+      </c>
+      <c r="AD37" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK37" t="n">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>